<commit_message>
Update Neoverse standalone availability for Neo-Fi items
</commit_message>
<xml_diff>
--- a/source/spreadsheets/Neoverse_for_Claude.xlsx
+++ b/source/spreadsheets/Neoverse_for_Claude.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmestes87/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC9F9180-AF0C-284E-85B9-C8C5CE32C145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3E2032-C3B2-774D-810B-1E82CAC5F7A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2300" yWindow="2400" windowWidth="26840" windowHeight="15680" xr2:uid="{BF29D5B1-F294-134E-8F7B-70D5B4D848F8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="143">
   <si>
     <t>Neoverse Interactive Edition</t>
   </si>
@@ -465,6 +465,9 @@
   </si>
   <si>
     <t>Billboards/External Live Video</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -1478,7 +1481,7 @@
         <v>6</v>
       </c>
       <c r="C48" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D48" t="s">
         <v>7</v>
@@ -1509,7 +1512,7 @@
         <v>6</v>
       </c>
       <c r="C50" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D50" t="s">
         <v>7</v>
@@ -1683,7 +1686,7 @@
         <v>6</v>
       </c>
       <c r="C62" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D62" t="s">
         <v>7</v>
@@ -1700,7 +1703,7 @@
         <v>6</v>
       </c>
       <c r="C63" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D63" t="s">
         <v>7</v>
@@ -2280,6 +2283,9 @@
       <c r="B109" t="s">
         <v>6</v>
       </c>
+      <c r="C109" t="s">
+        <v>142</v>
+      </c>
       <c r="D109" t="s">
         <v>7</v>
       </c>
@@ -2305,6 +2311,9 @@
       <c r="B111" t="s">
         <v>6</v>
       </c>
+      <c r="C111" t="s">
+        <v>142</v>
+      </c>
       <c r="D111" t="s">
         <v>7</v>
       </c>
@@ -2588,6 +2597,9 @@
       <c r="B135" t="s">
         <v>6</v>
       </c>
+      <c r="C135" t="s">
+        <v>142</v>
+      </c>
       <c r="D135" t="s">
         <v>7</v>
       </c>
@@ -2599,6 +2611,9 @@
       <c r="B136" t="s">
         <v>6</v>
       </c>
+      <c r="C136" t="s">
+        <v>142</v>
+      </c>
       <c r="D136" t="s">
         <v>7</v>
       </c>
@@ -2622,7 +2637,9 @@
       <c r="B138" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C138" s="2"/>
+      <c r="C138" s="2" t="s">
+        <v>142</v>
+      </c>
       <c r="D138" s="2"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Add SuperTouch requirement flag, new Neoverse features, Neo-Fi sync fix
</commit_message>
<xml_diff>
--- a/source/spreadsheets/Neoverse_for_Claude.xlsx
+++ b/source/spreadsheets/Neoverse_for_Claude.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmestes87/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3E2032-C3B2-774D-810B-1E82CAC5F7A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5EF43C-9524-E04E-A49E-5372E82AC6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2300" yWindow="2400" windowWidth="26840" windowHeight="15680" xr2:uid="{BF29D5B1-F294-134E-8F7B-70D5B4D848F8}"/>
+    <workbookView xWindow="40500" yWindow="2020" windowWidth="26840" windowHeight="15680" xr2:uid="{BF29D5B1-F294-134E-8F7B-70D5B4D848F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1 (2)" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="145">
   <si>
     <t>Neoverse Interactive Edition</t>
   </si>
@@ -468,6 +468,12 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Scheduler</t>
+  </si>
+  <si>
+    <t>Playlists</t>
   </si>
 </sst>
 </file>
@@ -854,7 +860,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7152A363-982E-1044-8657-DA2C0F17B383}">
-  <dimension ref="A1:E142"/>
+  <dimension ref="A1:E144"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.5" bestFit="1" customWidth="1"/>
@@ -879,26 +885,29 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>142</v>
       </c>
       <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
@@ -911,32 +920,42 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="2"/>
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="2"/>
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
@@ -950,7 +969,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
@@ -964,7 +983,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
@@ -978,7 +997,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
@@ -992,7 +1011,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
@@ -1005,20 +1024,22 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="2"/>
+      <c r="A12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
         <v>6</v>
@@ -1032,7 +1053,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
@@ -1046,7 +1067,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="B15" t="s">
         <v>6</v>
@@ -1060,661 +1081,649 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>142</v>
+      </c>
+      <c r="D17" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>142</v>
+      </c>
+      <c r="D18" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>13</v>
+      </c>
+      <c r="B32" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="2"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>18</v>
+      </c>
+      <c r="B37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" t="s">
+        <v>6</v>
+      </c>
+      <c r="D37" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>20</v>
       </c>
-      <c r="B16" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="B39" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
         <v>21</v>
       </c>
-      <c r="B17" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="B40" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>22</v>
       </c>
-      <c r="B18" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="B41" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" t="s">
+        <v>6</v>
+      </c>
+      <c r="D41" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
         <v>23</v>
       </c>
-      <c r="B19" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+      <c r="B42" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
+      <c r="B43" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="B44" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44" s="2"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
         <v>26</v>
       </c>
-      <c r="B22" t="s">
-        <v>6</v>
-      </c>
-      <c r="C22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="B45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>27</v>
       </c>
-      <c r="B23" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+      <c r="B46" t="s">
+        <v>6</v>
+      </c>
+      <c r="C46" t="s">
+        <v>6</v>
+      </c>
+      <c r="D46" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="2"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="B47" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" s="2"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
         <v>29</v>
       </c>
-      <c r="B25" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="B48" t="s">
+        <v>6</v>
+      </c>
+      <c r="C48" t="s">
+        <v>6</v>
+      </c>
+      <c r="D48" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>30</v>
       </c>
-      <c r="B26" t="s">
-        <v>6</v>
-      </c>
-      <c r="C26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
+      <c r="B49" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" t="s">
+        <v>6</v>
+      </c>
+      <c r="D49" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="2"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="B50" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D50" s="2"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
         <v>32</v>
       </c>
-      <c r="B28" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="B51" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" t="s">
+        <v>6</v>
+      </c>
+      <c r="D51" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
         <v>33</v>
       </c>
-      <c r="B29" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="B52" t="s">
+        <v>6</v>
+      </c>
+      <c r="C52" t="s">
+        <v>6</v>
+      </c>
+      <c r="D52" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>34</v>
       </c>
-      <c r="B30" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="B53" t="s">
+        <v>6</v>
+      </c>
+      <c r="C53" t="s">
+        <v>6</v>
+      </c>
+      <c r="D53" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>35</v>
       </c>
-      <c r="B31" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="B54" t="s">
+        <v>6</v>
+      </c>
+      <c r="C54" t="s">
+        <v>6</v>
+      </c>
+      <c r="D54" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>36</v>
       </c>
-      <c r="B32" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
+      <c r="B55" t="s">
+        <v>6</v>
+      </c>
+      <c r="C55" t="s">
+        <v>6</v>
+      </c>
+      <c r="D55" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="2"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="B56" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D56" s="2"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
         <v>38</v>
       </c>
-      <c r="B34" t="s">
-        <v>6</v>
-      </c>
-      <c r="C34" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="B57" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" t="s">
+        <v>6</v>
+      </c>
+      <c r="D57" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>39</v>
       </c>
-      <c r="B35" t="s">
-        <v>6</v>
-      </c>
-      <c r="C35" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+      <c r="B58" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" t="s">
+        <v>6</v>
+      </c>
+      <c r="D58" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>40</v>
       </c>
-      <c r="B36" t="s">
-        <v>6</v>
-      </c>
-      <c r="C36" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+      <c r="B59" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" t="s">
+        <v>6</v>
+      </c>
+      <c r="D59" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
         <v>41</v>
       </c>
-      <c r="B37" t="s">
-        <v>6</v>
-      </c>
-      <c r="C37" t="s">
-        <v>6</v>
-      </c>
-      <c r="D37" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+      <c r="B60" t="s">
+        <v>6</v>
+      </c>
+      <c r="C60" t="s">
+        <v>6</v>
+      </c>
+      <c r="D60" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
         <v>42</v>
       </c>
-      <c r="B38" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" t="s">
-        <v>6</v>
-      </c>
-      <c r="D38" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="B61" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" t="s">
+        <v>6</v>
+      </c>
+      <c r="D61" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
         <v>43</v>
       </c>
-      <c r="B39" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" t="s">
-        <v>6</v>
-      </c>
-      <c r="D39" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="B62" t="s">
+        <v>6</v>
+      </c>
+      <c r="C62" t="s">
+        <v>6</v>
+      </c>
+      <c r="D62" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
         <v>44</v>
       </c>
-      <c r="B40" t="s">
-        <v>6</v>
-      </c>
-      <c r="C40" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="B63" t="s">
+        <v>6</v>
+      </c>
+      <c r="C63" t="s">
+        <v>6</v>
+      </c>
+      <c r="D63" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
         <v>45</v>
-      </c>
-      <c r="B41" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" t="s">
-        <v>6</v>
-      </c>
-      <c r="D41" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>46</v>
-      </c>
-      <c r="B42" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" t="s">
-        <v>6</v>
-      </c>
-      <c r="D42" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>47</v>
-      </c>
-      <c r="B43" t="s">
-        <v>6</v>
-      </c>
-      <c r="C43" t="s">
-        <v>6</v>
-      </c>
-      <c r="D43" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>48</v>
-      </c>
-      <c r="B44" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" t="s">
-        <v>6</v>
-      </c>
-      <c r="D44" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>49</v>
-      </c>
-      <c r="B45" t="s">
-        <v>6</v>
-      </c>
-      <c r="C45" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>51</v>
-      </c>
-      <c r="B48" t="s">
-        <v>6</v>
-      </c>
-      <c r="C48" t="s">
-        <v>142</v>
-      </c>
-      <c r="D48" t="s">
-        <v>7</v>
-      </c>
-      <c r="E48" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>52</v>
-      </c>
-      <c r="B49" t="s">
-        <v>6</v>
-      </c>
-      <c r="C49" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>53</v>
-      </c>
-      <c r="B50" t="s">
-        <v>6</v>
-      </c>
-      <c r="C50" t="s">
-        <v>142</v>
-      </c>
-      <c r="D50" t="s">
-        <v>7</v>
-      </c>
-      <c r="E50" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>54</v>
-      </c>
-      <c r="B51" t="s">
-        <v>6</v>
-      </c>
-      <c r="C51" t="s">
-        <v>6</v>
-      </c>
-      <c r="D51" t="s">
-        <v>7</v>
-      </c>
-      <c r="E51" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>55</v>
-      </c>
-      <c r="B52" t="s">
-        <v>6</v>
-      </c>
-      <c r="C52" t="s">
-        <v>6</v>
-      </c>
-      <c r="D52" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>56</v>
-      </c>
-      <c r="B53" t="s">
-        <v>6</v>
-      </c>
-      <c r="C53" t="s">
-        <v>6</v>
-      </c>
-      <c r="D53" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>57</v>
-      </c>
-      <c r="B54" t="s">
-        <v>6</v>
-      </c>
-      <c r="C54" t="s">
-        <v>6</v>
-      </c>
-      <c r="D54" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>58</v>
-      </c>
-      <c r="B55" t="s">
-        <v>6</v>
-      </c>
-      <c r="C55" t="s">
-        <v>6</v>
-      </c>
-      <c r="D55" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>59</v>
-      </c>
-      <c r="B56" t="s">
-        <v>6</v>
-      </c>
-      <c r="C56" t="s">
-        <v>6</v>
-      </c>
-      <c r="D56" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>60</v>
-      </c>
-      <c r="B57" t="s">
-        <v>6</v>
-      </c>
-      <c r="C57" t="s">
-        <v>6</v>
-      </c>
-      <c r="D57" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>61</v>
-      </c>
-      <c r="B58" t="s">
-        <v>6</v>
-      </c>
-      <c r="C58" t="s">
-        <v>6</v>
-      </c>
-      <c r="D58" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
-        <v>62</v>
-      </c>
-      <c r="B59" t="s">
-        <v>6</v>
-      </c>
-      <c r="C59" t="s">
-        <v>6</v>
-      </c>
-      <c r="D59" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>63</v>
-      </c>
-      <c r="B60" t="s">
-        <v>6</v>
-      </c>
-      <c r="C60" t="s">
-        <v>6</v>
-      </c>
-      <c r="D60" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>64</v>
-      </c>
-      <c r="B61" t="s">
-        <v>6</v>
-      </c>
-      <c r="C61" t="s">
-        <v>6</v>
-      </c>
-      <c r="D61" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>65</v>
-      </c>
-      <c r="B62" t="s">
-        <v>6</v>
-      </c>
-      <c r="C62" t="s">
-        <v>142</v>
-      </c>
-      <c r="D62" t="s">
-        <v>7</v>
-      </c>
-      <c r="E62" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>66</v>
-      </c>
-      <c r="B63" t="s">
-        <v>6</v>
-      </c>
-      <c r="C63" t="s">
-        <v>142</v>
-      </c>
-      <c r="D63" t="s">
-        <v>7</v>
-      </c>
-      <c r="E63" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>67</v>
       </c>
       <c r="B64" t="s">
         <v>6</v>
@@ -1728,7 +1737,7 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="B65" t="s">
         <v>6</v>
@@ -1742,7 +1751,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="B66" t="s">
         <v>6</v>
@@ -1756,7 +1765,7 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="B67" t="s">
         <v>6</v>
@@ -1770,7 +1779,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="B68" t="s">
         <v>6</v>
@@ -2693,6 +2702,31 @@
         <v>6</v>
       </c>
       <c r="D142" s="2"/>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
+        <v>143</v>
+      </c>
+      <c r="B143" t="s">
+        <v>6</v>
+      </c>
+      <c r="C143" t="s">
+        <v>6</v>
+      </c>
+      <c r="D143" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A144" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>